<commit_message>
Address team review feedback (Phase 9)
- Elicitation plan: explain Observation/Survey are simulated; add SIM-OBS-01 and SIM-SURVEY-01 (not performed)
- Actor model: define 3 roles under Ban quan tri (AS-02/AS-04); TB-05a optional, TB-05b exception branch; note TB-06 split; PP-08 partial
- NFR-005: add backup retention and permission criteria (TBD)
- CQ-Q04: cite Bai 6.1 as reference for population fields
- Rewrite 17 RAW at stakeholder-need level, keep IDs, move original detail to Notes; sync 04/05/06 workbooks and docs
- Change workbook font Century Gothic -> Arial in 05/06
- Add docs/06_Team_Review_Response.md; remove references to nonexistent files; MoSCoW questions left for PO

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/04_Raw_Requirements.xlsx
+++ b/deliverables/04_Raw_Requirements.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="403">
   <si>
     <t>Wish ID</t>
   </si>
@@ -1121,6 +1121,108 @@
   </si>
   <si>
     <t>- Pain Points (PP-xx) xem docs/04_Interview_Report.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn lưu thông tin hộ gia đình tập trung và tránh trường hợp nhập trùng căn hộ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Dữ liệu cũ do Ban nhập (AS-08). Chi tiết ban đầu (trước Phase 9): Cho phép thêm hộ gia đình mới gồm số căn hộ, chủ hộ, diện tích căn hộ (m²), thông tin liên hệ; không cho trùng số căn hộ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn quản lý thông tin những người thuộc từng hộ và vẫn tra cứu được người đã rời đi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Có lưu số giấy tờ hay không: OQ-08; trường dữ liệu: AS-18. Chi tiết ban đầu (trước Phase 9): Cho phép thêm, sửa nhân khẩu trong hộ: họ tên, ngày sinh, giới tính, quan hệ với chủ hộ, giấy tờ tùy thân (nếu có); không xóa cứng nhân khẩu đã rời đi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn theo dõi các thay đổi nhân khẩu của từng hộ theo thời gian.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Danh sách loại biến động: OQ-13. Chi tiết ban đầu (trước Phase 9): Ghi nhận biến động nhân khẩu (chuyển đến, chuyển đi, sinh, mất…) kèm ngày và lý do; xem lịch sử biến động của từng hộ và từng nhân khẩu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn theo dõi tình trạng tạm trú/tạm vắng và thời hạn liên quan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Tình trạng cư trú: thường xuyên / tạm trú / tạm vắng (AS-18). Chi tiết ban đầu (trước Phase 9): Ghi nhận tạm trú và tạm vắng của nhân khẩu với thời gian bắt đầu, kết thúc và lý do; đánh dấu khi hết thời hạn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn tự quản lý các khoản thu và có thể thay đổi mức thu khi cần.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Không xóa khoản thu đã có giao dịch (AS-17); đơn giá cấu hình (AS-05). Chi tiết ban đầu (trước Phase 9): Cho phép tạo, xem, sửa, ngừng áp dụng khoản thu (phí dịch vụ, phí quản lý, khoản đóng góp) gồm tên, loại (bắt buộc / tự nguyện), kỳ thu hoặc đợt, đơn giá hoặc mức thu, hạn nộp; đơn giá cấu hình được.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn hệ thống hỗ trợ tính phí theo diện tích căn hộ để giảm tính toán thủ công.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Miễn/giảm chưa thuộc v1.0 (AS-14, OQ-02, C-02); kiot: OQ-03; thông báo từng hộ: OQ-06, AS-07. Chi tiết ban đầu (trước Phase 9): Hệ thống lập danh sách khoản phải thu của từng hộ theo kỳ và tự tính phí dịch vụ, phí quản lý theo diện tích × đơn giá; hiển thị rõ cách tính.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thủ quỹ muốn ghi nhận việc hộ nộp tiền, kể cả khi chỉ nộp một phần hoặc nhiều khoản cùng lúc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Ghi nhận cả người nộp hộ (nếu có). Hình thức nộp chỉ để ghi nhận (AS-12, OQ-09); phạt chậm nộp/nộp trước: OQ-05. Chi tiết ban đầu (trước Phase 9): Cho phép ghi nhận hộ nộp tiền: chọn hộ, khoản thu, số tiền, ngày nộp, hình thức nộp, người thu; hỗ trợ nộp một phần và nộp gộp nhiều khoản hoặc nhiều kỳ trong một lần.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thủ quỹ muốn xử lý được giao dịch thu ghi nhầm; phần truy vết thay đổi nằm ở RAW-025 và NFR-004.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Should. AS-17; chính sách tính lại: OQ-14. Chi tiết ban đầu (trước Phase 9): Cho phép sửa hoặc hủy giao dịch thu nhầm kèm lý do; không xóa cứng, lưu người thực hiện và thời điểm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thủ quỹ và BQT muốn tìm hộ gia đình theo số căn hộ và tên chủ hộ, kèm số tiền phải nộp; yêu cầu tốc độ nằm ở NFR-006.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Chi tiết ban đầu (trước Phase 9): Tìm hộ gia đình theo số căn hộ và tên chủ hộ; kết quả hiển thị nhanh kèm số tiền phải nộp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT và Thủ quỹ muốn tra cứu khoản thu và lịch sử đóng tiền của từng hộ theo nhiều tiêu chí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ưu tiên sơ bộ (gợi ý): Must. Chi tiết ban đầu (trước Phase 9): Tra cứu, lọc khoản thu và giao dịch theo hộ, khoản thu, kỳ, trạng thái nộp (đã nộp, còn thiếu, chưa nộp) và khoảng thời gian; xem công nợ và lịch sử nộp của một hộ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn tài khoản được bảo vệ an toàn và hạn chế truy cập trái phép.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại: Bảo mật. Ưu tiên sơ bộ (gợi ý): Must. Ngưỡng số lần sai là giả định cần xác thực. Chi tiết ban đầu (trước Phase 9): Xác thực an toàn: mật khẩu không lưu ở dạng rõ (băm), giới hạn số lần đăng nhập sai liên tiếp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi loại người dùng chỉ được thực hiện công việc phù hợp với trách nhiệm của mình.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại: Phân quyền. Ưu tiên sơ bộ (gợi ý): Should. C-01, AS-04, OQ-04. Chi tiết ban đầu (trước Phase 9): Phân quyền theo vai trò: tối thiểu phân biệt quản trị và người thu phí; chỉ quản trị được sửa hộ, nhân khẩu, khoản thu, đơn giá và tài khoản.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thông tin cá nhân nhạy cảm chỉ được người có thẩm quyền xem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại: Quyền riêng tư. Ưu tiên sơ bộ (gợi ý): Must. C-03, OQ-08, AS-10 (dữ liệu mẫu khi demo). Chi tiết ban đầu (trước Phase 9): Bảo vệ dữ liệu cá nhân: che bớt số giấy tờ khi hiển thị thường ngày; chỉ tài khoản có quyền mới xem đầy đủ và xuất dữ liệu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT muốn biết ai đã thay đổi dữ liệu quan trọng và thay đổi khi nào.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại: Truy vết. Ưu tiên sơ bộ (gợi ý): Should. Thời gian lưu giữ log: OQ-11. Chi tiết ban đầu (trước Phase 9): Audit log: ghi người thực hiện, thời điểm, loại thao tác, giá trị trước và sau cho việc thêm, sửa, hủy dữ liệu thu phí và nhân khẩu, và mỗi lần xuất dữ liệu; log không sửa hoặc xóa được qua giao diện.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQT lo mất dữ liệu và muốn có cách sao lưu, khôi phục khi có sự cố.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại: Độ tin cậy. Ưu tiên sơ bộ (gợi ý): Must (Ban coi là bắt buộc). Tần suất mặc định hằng ngày là giả định. Chi tiết ban đầu (trước Phase 9): Sao lưu và khôi phục dữ liệu: sao lưu tự động hoặc bằng một thao tác, có thể khôi phục khi cần.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thủ quỹ muốn việc tìm kiếm và mở danh sách không bị chậm khi dữ liệu tăng.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại: Hiệu năng. Ưu tiên sơ bộ (gợi ý): Should. Con số 3 giây và quy mô là giả định (AS-13, OQ-10). Chi tiết ban đầu (trước Phase 9): Hiệu năng: tìm kiếm và hiển thị danh sách trong tối đa 3 giây với quy mô vài trăm hộ, vài nghìn nhân khẩu và 2–3 người dùng đồng thời.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người dùng muốn giao diện tiếng Việt, dễ hiểu và thao tác thu phí đơn giản.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại: Khả năng sử dụng. Ưu tiên sơ bộ (gợi ý): Should. Số thao tác là giả định. Chi tiết ban đầu (trước Phase 9): Dễ dùng: giao diện tiếng Việt, tiền tệ VND hiển thị dễ đọc, thông báo lỗi rõ ràng; ghi nhận một lần nộp tiền không quá khoảng 5 thao tác chính; người không chuyên IT dùng được sau hướng dẫn ngắn.</t>
   </si>
 </sst>
 </file>
@@ -2394,7 +2496,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>171</v>
+        <v>369</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>160</v>
@@ -2409,7 +2511,7 @@
         <v>174</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>175</v>
+        <v>370</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -2481,7 +2583,7 @@
         <v>187</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>188</v>
+        <v>371</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>160</v>
@@ -2496,7 +2598,7 @@
         <v>191</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>192</v>
+        <v>372</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -2510,7 +2612,7 @@
         <v>187</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>193</v>
+        <v>373</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>160</v>
@@ -2525,7 +2627,7 @@
         <v>191</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>196</v>
+        <v>374</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -2539,7 +2641,7 @@
         <v>187</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>198</v>
+        <v>375</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>160</v>
@@ -2554,7 +2656,7 @@
         <v>191</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>201</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -2597,7 +2699,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>209</v>
+        <v>377</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>160</v>
@@ -2612,7 +2714,7 @@
         <v>212</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>213</v>
+        <v>378</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2626,7 +2728,7 @@
         <v>214</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>215</v>
+        <v>379</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>160</v>
@@ -2641,7 +2743,7 @@
         <v>212</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>218</v>
+        <v>380</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2684,7 +2786,7 @@
         <v>224</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>225</v>
+        <v>381</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>160</v>
@@ -2699,7 +2801,7 @@
         <v>228</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>229</v>
+        <v>382</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2742,7 +2844,7 @@
         <v>236</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>237</v>
+        <v>383</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>160</v>
@@ -2757,7 +2859,7 @@
         <v>228</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>240</v>
+        <v>384</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -2771,7 +2873,7 @@
         <v>242</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>243</v>
+        <v>385</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>160</v>
@@ -2786,7 +2888,7 @@
         <v>246</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>169</v>
+        <v>386</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -2829,7 +2931,7 @@
         <v>214</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>253</v>
+        <v>387</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>160</v>
@@ -2844,7 +2946,7 @@
         <v>246</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>169</v>
+        <v>388</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -2945,7 +3047,7 @@
         <v>158</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>271</v>
+        <v>389</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>272</v>
@@ -2960,7 +3062,7 @@
         <v>274</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>275</v>
+        <v>390</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -2974,7 +3076,7 @@
         <v>158</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>276</v>
+        <v>391</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>272</v>
@@ -2989,7 +3091,7 @@
         <v>274</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>279</v>
+        <v>392</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -3003,7 +3105,7 @@
         <v>281</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>282</v>
+        <v>393</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>272</v>
@@ -3018,7 +3120,7 @@
         <v>274</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>285</v>
+        <v>394</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -3032,7 +3134,7 @@
         <v>287</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>288</v>
+        <v>395</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>272</v>
@@ -3047,7 +3149,7 @@
         <v>274</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>291</v>
+        <v>396</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -3061,7 +3163,7 @@
         <v>8</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>292</v>
+        <v>397</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>272</v>
@@ -3076,7 +3178,7 @@
         <v>274</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>294</v>
+        <v>398</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -3090,7 +3192,7 @@
         <v>58</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>296</v>
+        <v>399</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>272</v>
@@ -3105,7 +3207,7 @@
         <v>274</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>299</v>
+        <v>400</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -3119,7 +3221,7 @@
         <v>224</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>301</v>
+        <v>401</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>272</v>
@@ -3134,7 +3236,7 @@
         <v>274</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>304</v>
+        <v>402</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>